<commit_message>
Update department evaluation tool with DEF column data population
Key features implemented:
- Modified process_cadres.py to populate columns D, E, F in results summary table with考核基数 (evaluation base), 外派干部人数 (external cadre count), and 评优名额 (excellence quota)
- Enhanced department mapping logic to maintain consistency between summary and annual cadre tables
- Updated .gitignore with comprehensive file exclusion patterns for Python projects, IDE files, and compressed archives
- Integrated statistical calculations for department evaluation metrics including base counts excluding external cadres

The tool now automatically fills the DEF columns in the summary sheet with calculated evaluation statistics based on departmental cadre data and performance ratings.
</commit_message>
<xml_diff>
--- a/公司党委管理四级正（副）干部综合考核评价情况汇总表_已填充.xlsx
+++ b/公司党委管理四级正（副）干部综合考核评价情况汇总表_已填充.xlsx
@@ -1808,10 +1808,18 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D6" s="63" t="n"/>
-      <c r="E6" s="63" t="n"/>
-      <c r="F6" s="63" t="n"/>
-      <c r="G6" s="63" t="n"/>
+      <c r="D6" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H6" s="62" t="n"/>
       <c r="I6" s="64" t="n"/>
       <c r="J6" s="88" t="n"/>
@@ -1854,10 +1862,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D7" s="63" t="n"/>
-      <c r="E7" s="63" t="n"/>
-      <c r="F7" s="63" t="n"/>
-      <c r="G7" s="63" t="n"/>
+      <c r="D7" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H7" s="62" t="n"/>
       <c r="I7" s="64" t="n"/>
       <c r="J7" s="64" t="n"/>
@@ -1900,10 +1916,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D8" s="63" t="n"/>
-      <c r="E8" s="63" t="n"/>
-      <c r="F8" s="63" t="n"/>
-      <c r="G8" s="63" t="n"/>
+      <c r="D8" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="62" t="n"/>
       <c r="I8" s="88" t="n"/>
       <c r="J8" s="88" t="n"/>
@@ -1946,10 +1970,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D9" s="63" t="n"/>
-      <c r="E9" s="63" t="n"/>
-      <c r="F9" s="63" t="n"/>
-      <c r="G9" s="63" t="n"/>
+      <c r="D9" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="62" t="n"/>
       <c r="I9" s="64" t="n"/>
       <c r="J9" s="88" t="n"/>
@@ -1992,10 +2024,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D10" s="63" t="n"/>
-      <c r="E10" s="63" t="n"/>
-      <c r="F10" s="63" t="n"/>
-      <c r="G10" s="63" t="n"/>
+      <c r="D10" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H10" s="62" t="n"/>
       <c r="I10" s="64" t="n"/>
       <c r="J10" s="88" t="n"/>
@@ -2078,10 +2118,18 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D12" s="63" t="n"/>
-      <c r="E12" s="63" t="n"/>
-      <c r="F12" s="63" t="n"/>
-      <c r="G12" s="63" t="n"/>
+      <c r="D12" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H12" s="62" t="n"/>
       <c r="I12" s="64" t="n"/>
       <c r="J12" s="64" t="n"/>
@@ -2124,10 +2172,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D13" s="63" t="n"/>
-      <c r="E13" s="63" t="n"/>
-      <c r="F13" s="63" t="n"/>
-      <c r="G13" s="63" t="n"/>
+      <c r="D13" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H13" s="62" t="n"/>
       <c r="I13" s="64" t="n"/>
       <c r="J13" s="88" t="n"/>
@@ -2170,10 +2226,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D14" s="63" t="n"/>
-      <c r="E14" s="63" t="n"/>
-      <c r="F14" s="63" t="n"/>
-      <c r="G14" s="63" t="n"/>
+      <c r="D14" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H14" s="62" t="n"/>
       <c r="I14" s="64" t="n"/>
       <c r="J14" s="88" t="n"/>
@@ -2216,10 +2280,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D15" s="63" t="n"/>
-      <c r="E15" s="63" t="n"/>
-      <c r="F15" s="63" t="n"/>
-      <c r="G15" s="63" t="n"/>
+      <c r="D15" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H15" s="62" t="n"/>
       <c r="I15" s="64" t="n"/>
       <c r="J15" s="88" t="n"/>
@@ -2302,10 +2374,18 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D17" s="63" t="n"/>
-      <c r="E17" s="63" t="n"/>
-      <c r="F17" s="63" t="n"/>
-      <c r="G17" s="63" t="n"/>
+      <c r="D17" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H17" s="62" t="n"/>
       <c r="I17" s="64" t="n"/>
       <c r="J17" s="88" t="n"/>
@@ -2348,10 +2428,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D18" s="63" t="n"/>
-      <c r="E18" s="63" t="n"/>
-      <c r="F18" s="63" t="n"/>
-      <c r="G18" s="63" t="n"/>
+      <c r="D18" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H18" s="62" t="n"/>
       <c r="I18" s="64" t="n"/>
       <c r="J18" s="88" t="n"/>
@@ -2394,10 +2482,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D19" s="63" t="n"/>
-      <c r="E19" s="63" t="n"/>
-      <c r="F19" s="63" t="n"/>
-      <c r="G19" s="63" t="n"/>
+      <c r="D19" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H19" s="62" t="n"/>
       <c r="I19" s="64" t="n"/>
       <c r="J19" s="88" t="n"/>
@@ -2440,10 +2536,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D20" s="63" t="n"/>
-      <c r="E20" s="63" t="n"/>
-      <c r="F20" s="63" t="n"/>
-      <c r="G20" s="63" t="n"/>
+      <c r="D20" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H20" s="62" t="n"/>
       <c r="I20" s="64" t="n"/>
       <c r="J20" s="88" t="n"/>
@@ -2526,10 +2630,18 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D22" s="52" t="n"/>
-      <c r="E22" s="52" t="n"/>
-      <c r="F22" s="52" t="n"/>
-      <c r="G22" s="52" t="n"/>
+      <c r="D22" s="52" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="52" t="n">
+        <v>0</v>
+      </c>
       <c r="H22" s="57" t="n"/>
       <c r="I22" s="87" t="n"/>
       <c r="J22" s="87" t="n"/>
@@ -2572,10 +2684,18 @@
           <t>/</t>
         </is>
       </c>
-      <c r="D23" s="52" t="n"/>
-      <c r="E23" s="52" t="n"/>
-      <c r="F23" s="52" t="n"/>
-      <c r="G23" s="52" t="n"/>
+      <c r="D23" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="52" t="n">
+        <v>0</v>
+      </c>
       <c r="H23" s="57" t="n"/>
       <c r="I23" s="87" t="n"/>
       <c r="J23" s="87" t="n"/>
@@ -2618,10 +2738,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D24" s="52" t="n"/>
-      <c r="E24" s="52" t="n"/>
-      <c r="F24" s="52" t="n"/>
-      <c r="G24" s="52" t="n"/>
+      <c r="D24" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="52" t="n">
+        <v>0</v>
+      </c>
       <c r="H24" s="57" t="n"/>
       <c r="I24" s="87" t="n"/>
       <c r="J24" s="87" t="n"/>
@@ -2664,10 +2792,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D25" s="52" t="n"/>
-      <c r="E25" s="52" t="n"/>
-      <c r="F25" s="52" t="n"/>
-      <c r="G25" s="52" t="n"/>
+      <c r="D25" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="52" t="n">
+        <v>0</v>
+      </c>
       <c r="H25" s="57" t="n"/>
       <c r="I25" s="87" t="n"/>
       <c r="J25" s="87" t="n"/>
@@ -2710,10 +2846,18 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D26" s="52" t="n"/>
-      <c r="E26" s="52" t="n"/>
-      <c r="F26" s="52" t="n"/>
-      <c r="G26" s="52" t="n"/>
+      <c r="D26" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="52" t="n">
+        <v>0</v>
+      </c>
       <c r="H26" s="57" t="n"/>
       <c r="I26" s="87" t="n"/>
       <c r="J26" s="87" t="n"/>
@@ -2796,10 +2940,18 @@
           <t>优秀</t>
         </is>
       </c>
-      <c r="D28" s="63" t="n"/>
-      <c r="E28" s="63" t="n"/>
-      <c r="F28" s="63" t="n"/>
-      <c r="G28" s="63" t="n"/>
+      <c r="D28" s="63" t="n">
+        <v>23</v>
+      </c>
+      <c r="E28" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="G28" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H28" s="62" t="n"/>
       <c r="I28" s="64" t="n"/>
       <c r="J28" s="88" t="n"/>
@@ -2842,10 +2994,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D29" s="63" t="n"/>
-      <c r="E29" s="63" t="n"/>
-      <c r="F29" s="63" t="n"/>
-      <c r="G29" s="63" t="n"/>
+      <c r="D29" s="63" t="n">
+        <v>26</v>
+      </c>
+      <c r="E29" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H29" s="62" t="n"/>
       <c r="I29" s="64" t="n"/>
       <c r="J29" s="64" t="n"/>
@@ -2888,10 +3048,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D30" s="63" t="n"/>
-      <c r="E30" s="63" t="n"/>
-      <c r="F30" s="63" t="n"/>
-      <c r="G30" s="63" t="n"/>
+      <c r="D30" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="62" t="n"/>
       <c r="I30" s="88" t="n"/>
       <c r="J30" s="88" t="n"/>
@@ -2934,10 +3102,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D31" s="63" t="n"/>
-      <c r="E31" s="63" t="n"/>
-      <c r="F31" s="63" t="n"/>
-      <c r="G31" s="63" t="n"/>
+      <c r="D31" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E31" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H31" s="62" t="n"/>
       <c r="I31" s="64" t="n"/>
       <c r="J31" s="88" t="n"/>
@@ -2980,10 +3156,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D32" s="63" t="n"/>
-      <c r="E32" s="63" t="n"/>
-      <c r="F32" s="63" t="n"/>
-      <c r="G32" s="63" t="n"/>
+      <c r="D32" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H32" s="62" t="n"/>
       <c r="I32" s="64" t="n"/>
       <c r="J32" s="88" t="n"/>
@@ -3026,10 +3210,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D33" s="63" t="n"/>
-      <c r="E33" s="63" t="n"/>
-      <c r="F33" s="63" t="n"/>
-      <c r="G33" s="63" t="n"/>
+      <c r="D33" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H33" s="62" t="n"/>
       <c r="I33" s="64" t="n"/>
       <c r="J33" s="88" t="n"/>
@@ -3072,10 +3264,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D34" s="63" t="n"/>
-      <c r="E34" s="63" t="n"/>
-      <c r="F34" s="63" t="n"/>
-      <c r="G34" s="63" t="n"/>
+      <c r="D34" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H34" s="62" t="n"/>
       <c r="I34" s="64" t="n"/>
       <c r="J34" s="64" t="n"/>
@@ -3122,10 +3322,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D35" s="63" t="n"/>
-      <c r="E35" s="63" t="n"/>
-      <c r="F35" s="63" t="n"/>
-      <c r="G35" s="63" t="n"/>
+      <c r="D35" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="E35" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H35" s="62" t="n"/>
       <c r="I35" s="64" t="n"/>
       <c r="J35" s="88" t="n"/>
@@ -3168,10 +3376,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D36" s="63" t="n"/>
-      <c r="E36" s="63" t="n"/>
-      <c r="F36" s="63" t="n"/>
-      <c r="G36" s="63" t="n"/>
+      <c r="D36" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H36" s="62" t="n"/>
       <c r="I36" s="64" t="n"/>
       <c r="J36" s="88" t="n"/>
@@ -3214,10 +3430,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D37" s="63" t="n"/>
-      <c r="E37" s="63" t="n"/>
-      <c r="F37" s="63" t="n"/>
-      <c r="G37" s="63" t="n"/>
+      <c r="D37" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="E37" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H37" s="62" t="n"/>
       <c r="I37" s="64" t="n"/>
       <c r="J37" s="88" t="n"/>
@@ -3260,10 +3484,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D38" s="63" t="n"/>
-      <c r="E38" s="63" t="n"/>
-      <c r="F38" s="63" t="n"/>
-      <c r="G38" s="63" t="n"/>
+      <c r="D38" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E38" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H38" s="62" t="n"/>
       <c r="I38" s="64" t="n"/>
       <c r="J38" s="88" t="n"/>
@@ -3346,10 +3578,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D40" s="63" t="n"/>
-      <c r="E40" s="63" t="n"/>
-      <c r="F40" s="63" t="n"/>
-      <c r="G40" s="63" t="n"/>
+      <c r="D40" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="E40" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H40" s="62" t="n"/>
       <c r="I40" s="88" t="n"/>
       <c r="J40" s="89" t="n"/>
@@ -3392,10 +3632,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D41" s="63" t="n"/>
-      <c r="E41" s="63" t="n"/>
-      <c r="F41" s="63" t="n"/>
-      <c r="G41" s="63" t="n"/>
+      <c r="D41" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="E41" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H41" s="62" t="n"/>
       <c r="I41" s="88" t="n"/>
       <c r="J41" s="89" t="n"/>
@@ -3438,10 +3686,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D42" s="63" t="n"/>
-      <c r="E42" s="63" t="n"/>
-      <c r="F42" s="63" t="n"/>
-      <c r="G42" s="63" t="n"/>
+      <c r="D42" s="63" t="n">
+        <v>17</v>
+      </c>
+      <c r="E42" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H42" s="62" t="n"/>
       <c r="I42" s="64" t="n"/>
       <c r="J42" s="89" t="n"/>
@@ -3488,10 +3744,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D43" s="63" t="n"/>
-      <c r="E43" s="63" t="n"/>
-      <c r="F43" s="63" t="n"/>
-      <c r="G43" s="63" t="n"/>
+      <c r="D43" s="63" t="n">
+        <v>12</v>
+      </c>
+      <c r="E43" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H43" s="62" t="n"/>
       <c r="I43" s="64" t="n"/>
       <c r="J43" s="89" t="n"/>
@@ -3534,10 +3798,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D44" s="63" t="n"/>
-      <c r="E44" s="63" t="n"/>
-      <c r="F44" s="63" t="n"/>
-      <c r="G44" s="63" t="n"/>
+      <c r="D44" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H44" s="62" t="n"/>
       <c r="I44" s="89" t="n"/>
       <c r="J44" s="89" t="n"/>
@@ -3620,10 +3892,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D46" s="63" t="n"/>
-      <c r="E46" s="63" t="n"/>
-      <c r="F46" s="63" t="n"/>
-      <c r="G46" s="63" t="n"/>
+      <c r="D46" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H46" s="62" t="n"/>
       <c r="I46" s="88" t="n"/>
       <c r="J46" s="89" t="n"/>
@@ -3666,10 +3946,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D47" s="63" t="n"/>
-      <c r="E47" s="63" t="n"/>
-      <c r="F47" s="63" t="n"/>
-      <c r="G47" s="63" t="n"/>
+      <c r="D47" s="63" t="n">
+        <v>9</v>
+      </c>
+      <c r="E47" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H47" s="62" t="n"/>
       <c r="I47" s="64" t="n"/>
       <c r="J47" s="89" t="n"/>
@@ -3712,10 +4000,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D48" s="63" t="n"/>
-      <c r="E48" s="63" t="n"/>
-      <c r="F48" s="63" t="n"/>
-      <c r="G48" s="63" t="n"/>
+      <c r="D48" s="63" t="n">
+        <v>11</v>
+      </c>
+      <c r="E48" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H48" s="62" t="n"/>
       <c r="I48" s="63" t="n"/>
       <c r="J48" s="89" t="n"/>
@@ -3758,10 +4054,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D49" s="63" t="n"/>
-      <c r="E49" s="63" t="n"/>
-      <c r="F49" s="63" t="n"/>
-      <c r="G49" s="63" t="n"/>
+      <c r="D49" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="E49" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G49" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H49" s="62" t="n"/>
       <c r="I49" s="64" t="n"/>
       <c r="J49" s="89" t="n"/>
@@ -3844,10 +4148,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D51" s="63" t="n"/>
-      <c r="E51" s="63" t="n"/>
-      <c r="F51" s="63" t="n"/>
-      <c r="G51" s="63" t="n"/>
+      <c r="D51" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H51" s="62" t="n"/>
       <c r="I51" s="63" t="n"/>
       <c r="J51" s="89" t="n"/>
@@ -3890,10 +4202,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D52" s="63" t="n"/>
-      <c r="E52" s="63" t="n"/>
-      <c r="F52" s="63" t="n"/>
-      <c r="G52" s="63" t="n"/>
+      <c r="D52" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E52" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G52" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H52" s="62" t="n"/>
       <c r="I52" s="63" t="n"/>
       <c r="J52" s="89" t="n"/>
@@ -3936,10 +4256,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D53" s="63" t="n"/>
-      <c r="E53" s="63" t="n"/>
-      <c r="F53" s="63" t="n"/>
-      <c r="G53" s="63" t="n"/>
+      <c r="D53" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H53" s="62" t="n"/>
       <c r="I53" s="63" t="n"/>
       <c r="J53" s="89" t="n"/>
@@ -3982,10 +4310,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D54" s="63" t="n"/>
-      <c r="E54" s="63" t="n"/>
-      <c r="F54" s="63" t="n"/>
-      <c r="G54" s="63" t="n"/>
+      <c r="D54" s="63" t="n">
+        <v>13</v>
+      </c>
+      <c r="E54" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G54" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H54" s="62" t="n"/>
       <c r="I54" s="64" t="n"/>
       <c r="J54" s="89" t="n"/>
@@ -4064,10 +4400,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D56" s="63" t="n"/>
-      <c r="E56" s="63" t="n"/>
-      <c r="F56" s="63" t="n"/>
-      <c r="G56" s="63" t="n"/>
+      <c r="D56" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H56" s="62" t="n"/>
       <c r="I56" s="88" t="n"/>
       <c r="J56" s="89" t="n"/>
@@ -4156,10 +4500,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D58" s="63" t="n"/>
-      <c r="E58" s="63" t="n"/>
-      <c r="F58" s="63" t="n"/>
-      <c r="G58" s="63" t="n"/>
+      <c r="D58" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H58" s="62" t="n"/>
       <c r="I58" s="88" t="n"/>
       <c r="J58" s="89" t="n"/>
@@ -4202,10 +4554,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D59" s="63" t="n"/>
-      <c r="E59" s="63" t="n"/>
-      <c r="F59" s="63" t="n"/>
-      <c r="G59" s="63" t="n"/>
+      <c r="D59" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E59" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H59" s="62" t="n"/>
       <c r="I59" s="64" t="n"/>
       <c r="J59" s="89" t="n"/>
@@ -4248,10 +4608,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D60" s="63" t="n"/>
-      <c r="E60" s="63" t="n"/>
-      <c r="F60" s="63" t="n"/>
-      <c r="G60" s="63" t="n"/>
+      <c r="D60" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E60" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H60" s="62" t="n"/>
       <c r="I60" s="63" t="n"/>
       <c r="J60" s="89" t="n"/>
@@ -4426,10 +4794,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D64" s="63" t="n"/>
-      <c r="E64" s="63" t="n"/>
-      <c r="F64" s="63" t="n"/>
-      <c r="G64" s="63" t="n"/>
+      <c r="D64" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H64" s="62" t="n"/>
       <c r="I64" s="63" t="n"/>
       <c r="J64" s="89" t="n"/>
@@ -4472,10 +4848,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D65" s="63" t="n"/>
-      <c r="E65" s="63" t="n"/>
-      <c r="F65" s="63" t="n"/>
-      <c r="G65" s="63" t="n"/>
+      <c r="D65" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="E65" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H65" s="62" t="n"/>
       <c r="I65" s="63" t="n"/>
       <c r="J65" s="89" t="n"/>
@@ -4518,10 +4902,18 @@
           <t>良好</t>
         </is>
       </c>
-      <c r="D66" s="63" t="n"/>
-      <c r="E66" s="63" t="n"/>
-      <c r="F66" s="63" t="n"/>
-      <c r="G66" s="63" t="n"/>
+      <c r="D66" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="63" t="n">
+        <v>0</v>
+      </c>
       <c r="H66" s="62" t="n"/>
       <c r="I66" s="63" t="n"/>
       <c r="J66" s="89" t="n"/>
@@ -4602,10 +4994,18 @@
         </is>
       </c>
       <c r="C68" s="72" t="n"/>
-      <c r="D68" s="72" t="n"/>
-      <c r="E68" s="72" t="n"/>
-      <c r="F68" s="72" t="n"/>
-      <c r="G68" s="72" t="n"/>
+      <c r="D68" s="72" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="72" t="n">
+        <v>0</v>
+      </c>
       <c r="H68" s="73" t="n"/>
       <c r="I68" s="73" t="n"/>
       <c r="J68" s="73" t="n"/>
@@ -4714,6 +5114,7 @@
       <c r="S70" s="79" t="n"/>
       <c r="T70" s="79" t="n"/>
     </row>
+    <row r="71"/>
     <row r="72" ht="44" customHeight="1" s="4">
       <c r="C72" s="76" t="inlineStr">
         <is>
@@ -4794,6 +5195,8 @@
       <c r="S73" s="79" t="n"/>
       <c r="T73" s="79" t="n"/>
     </row>
+    <row r="74"/>
+    <row r="75"/>
     <row r="76" ht="20.25" customHeight="1" s="4">
       <c r="D76" s="48" t="n"/>
       <c r="E76" s="48" t="n"/>

</xml_diff>